<commit_message>
Mandate 08:15: UNSW Bengaluru English withdrawal paste and bounded fee target-list window pastes (not applied; dry runs passed); v1 proposal marked superseded
</commit_message>
<xml_diff>
--- a/docs/platform/reports/2026-10-27/AU-fee-target-list-proposal-2026-10-27.xlsx
+++ b/docs/platform/reports/2026-10-27/AU-fee-target-list-proposal-2026-10-27.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -434,139 +434,279 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Fee-schedule pages refused by the Firecrawl target list: proposal for a Platform Admin decision (not applied)</t>
+          <t>VERSION 2 (27 Oct 2026 08:3x, Platform Admin mandate 08:15 item 5). Version 1 below is superseded and NOT authorised.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pastes: PASTE-20261027-fee-target-window-open.sql (part A) and PASTE-20261027-fee-target-window-close.sql (part B). Not applied; for separate authority.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Prepared 27 Oct 2026 07:1x from the live database (project fxcwkweaxjtknorudmwp), under the Platform Admin mandate of 27 Oct 05:46 (Priority 2B).</t>
+          <t>Rolled-back dry run of A then B on live: passed (run 40404051903): 42 providers included then closed, 54 pages back to the reader, 0 credits spent in the dry run.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>The 26 Oct AU fee-schedule wave found 284 pages: 167 read (12 with fee rows, 155 without) and 117 failed (110 'target_list_refused', 7 'no content').</t>
+          <t>Why not a 54-reads-only version: the fee-schedule lane reads every page through Firecrawl with no direct read first, and Firecrawl eligibility is per provider.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>A 'target_list_refused' page could not be read directly (blocked) and the scraper refused it because the provider is not on the Firecrawl target list.</t>
+          <t xml:space="preserve">  No existing control limits Firecrawl to named pages. A worker change (read directly first, as the entry-matrix lane does) would read most of these pages</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  at zero credits; it is named here as an alternative for a decision and is not built (not authorised by this mandate).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>What this file proposes</t>
+          <t>Bounded window instead: A adds the 42 providers and returns the 54 pages; B (after the pages settle, or 24 hours) removes them and reports the spend.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Of the 110 refused pages (66 providers), 54 are proposed for one read (Candidate). They belong to 42 providers, which hold 400 active courses with no admitted provider tuition.</t>
+          <t>Cross-lane inventory while the window is open (live 27 Oct 08:3x) and worst case for 24 hours:</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  The others are excluded: PDF files (PDF work is not authorised), duplicate addresses, or pages that are not tuition schedules (policies, payment methods, tuition protection, FEE-HELP, research, cost of living).</t>
+          <t xml:space="preserve">  fee-schedule pages (the purpose): 54 pages x 3 attempts x 1 credit = 162</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Nothing has been changed. The paste file PASTE-20261027-fee-target-list-proposal.sql applies it only if run by the Platform Admin; it is count-guarded and stops if the live state differs.</t>
+          <t xml:space="preserve">  course-page search, queued items: 83 x 3 attempts x 2 credits = 498</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  course pages needing the scraper (blocked 5, needs rendering 22, fetch failed 18): 45 x 3 x 1 = 135</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Estimated cost</t>
+          <t xml:space="preserve">  course-list re-reads: 10 lists x 10 pages x 1 = 100</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Firecrawl: 1 credit per page read on the basic proxy; 54 credits expected, at most 162 if every page uses all 3 attempts.</t>
+          <t xml:space="preserve">  site maps (discovery 42, source-find 17): 59 x 2 = 118</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AI fee reader: about US$0.0036 per page (the 26 Oct wave: US$0.60 for 167 pages), about US$0.19.</t>
+          <t xml:space="preserve">  english/calendar pages: 0 (all failed or read; none returns to a reader without a person); scholarships, central maps, site checks: 0 extra (already bypass the list)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Hidden effect, the main cost risk: the target list is per provider, not per purpose. Adding these providers also lets other lanes (course-page search and reads, scholarships, central pages) spend Firecrawl credits on them within their own daily shares.</t>
+          <t xml:space="preserve">  WORST CASE: 1,013 credits; at most 199 pages scraped, 249 searches, 118 maps. Expected about 54-120 credits. Hard ceiling still: daily budget 25,000 and lane caps.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Testable: part B sums pipeline.coverage_vendor_usage for these providers since part A and records it against 1,013 (within_bound true/false).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Expected yield (from the 26 Oct wave, not a promise)</t>
+          <t>Coverage versus admissions (kept separate):</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  44 of 167 read pages gave fee rows; 121 courses were admitted and 104 sent to Layer 4 review. At that rate the 54 candidates would give rows on about 14 pages.</t>
+          <t xml:space="preserve">  courses at these 42 providers with no provider tuition, covered by a source: 400 (not admissions);</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  expected admitted tuition values: about 40 courses, plus about 30 to Layer 4 review (26 Oct wave rate: 44 of 167 read pages gave rows; 121 admitted, 104 review).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Exclusions kept: 22 PDFs, 33 non-tuition pages, 1 duplicate address.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  'MIT - Melbourne Institute of Technology' and 'Melbourne Institute of Technology' are two provider records with the same fee page: an identity question for the Platform Admin, not resolved here.</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>---- Version 1 (07:1x, superseded) ----</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Fee-schedule pages refused by the Firecrawl target list: proposal for a Platform Admin decision (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Prepared 27 Oct 2026 07:1x from the live database (project fxcwkweaxjtknorudmwp), under the Platform Admin mandate of 27 Oct 05:46 (Priority 2B).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>The 26 Oct AU fee-schedule wave found 284 pages: 167 read (12 with fee rows, 155 without) and 117 failed (110 'target_list_refused', 7 'no content').</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>A 'target_list_refused' page could not be read directly (blocked) and the scraper refused it because the provider is not on the Firecrawl target list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>What this file proposes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Of the 110 refused pages (66 providers), 54 are proposed for one read (Candidate). They belong to 42 providers, which hold 400 active courses with no admitted provider tuition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The others are excluded: PDF files (PDF work is not authorised), duplicate addresses, or pages that are not tuition schedules (policies, payment methods, tuition protection, FEE-HELP, research, cost of living).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Nothing has been changed. The paste file PASTE-20261027-fee-target-list-proposal.sql applies it only if run by the Platform Admin; it is count-guarded and stops if the live state differs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Estimated cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Firecrawl: 1 credit per page read on the basic proxy; 54 credits expected, at most 162 if every page uses all 3 attempts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AI fee reader: about US$0.0036 per page (the 26 Oct wave: US$0.60 for 167 pages), about US$0.19.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Hidden effect, the main cost risk: the target list is per provider, not per purpose. Adding these providers also lets other lanes (course-page search and reads, scholarships, central pages) spend Firecrawl credits on them within their own daily shares.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Expected yield (from the 26 Oct wave, not a promise)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  44 of 167 read pages gave fee rows; 121 courses were admitted and 104 sent to Layer 4 review. At that rate the 54 candidates would give rows on about 14 pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  'MIT - Melbourne Institute of Technology' and 'Melbourne Institute of Technology' are two provider records with the same fee page: an identity question for the Platform Admin, not resolved here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Victoria University is on the list for its fee pages only (its entry-matrix lane stays excluded).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t xml:space="preserve">  12 older pages (12–22 Oct) failed for the same reason; they are listed on their own sheet for completeness and are not in the proposal.</t>
         </is>

</xml_diff>